<commit_message>
data: 2026-07-02 일별 수집
</commit_message>
<xml_diff>
--- a/data/daily/2026-07/2026-07-02.xlsx
+++ b/data/daily/2026-07/2026-07-02.xlsx
@@ -20,13 +20,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,32 +440,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -530,7 +542,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 10입(7+3) - 스페셜 기프트 에디션 (공식수입)</t>
+          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 10입 - 슬리브 기프트 에디션 (공식수입)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -870,7 +882,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>19,900원</t>
+          <t>31,500원</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -972,7 +984,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -980,29 +992,29 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>식물성 멜라토닌 1mg 구미 젤리 멜라메이트 1박스 (20구미) 수험생/직장인 선물</t>
+          <t>대한민국 NO.1 김종국 트리플아르기닌 6200 (30포) + 아르기닌 추가 증정</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CJ웰케어</t>
+          <t>익스트림</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>9,900원</t>
+          <t>45,000원</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/11190137</t>
+          <t>https://gift.kakao.com/product/7417420</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1010,22 +1022,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>대한민국 NO.1 김종국 트리플아르기닌 6200 (30포) + 아르기닌 추가 증정</t>
+          <t>식물성 멜라토닌 1mg 구미 젤리 멜라메이트 1박스 (20구미) 수험생/직장인 선물</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>익스트림</t>
+          <t>CJ웰케어</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>45,000원</t>
+          <t>9,900원</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/7417420</t>
+          <t>https://gift.kakao.com/product/11190137</t>
         </is>
       </c>
     </row>
@@ -1073,41 +1085,41 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -1116,7 +1128,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1124,29 +1136,29 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>밀크씨슬 30정 30일분</t>
+          <t>[김종국 PICK] 익스트림 아르기닌 에너지온 2개입 2일분</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>익스트림</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>1,500원</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000134&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=987253277&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>홍삼/인삼</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1154,29 +1166,29 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>하루한포 6년근 고려홍삼 5포 5일분</t>
+          <t>푸응 7days 팻버닝 21캡슐</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>휴럼</t>
+          <t>닥터블릿</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2,000원</t>
+          <t>5,000원</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=919157053&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=613602085&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>마그네슘</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1184,29 +1196,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>마그네슘 30정 30일분</t>
+          <t>[다영 PICK] 셀트리온 다이어트 한 잔 슬림 S 프레소 10포 5일분</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3,000원</t>
+          <t>2,000원</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000128&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=944863413&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>루테인/눈건강</t>
+          <t>피부/미용</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1214,7 +1226,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>식물성 뉴티지 오메가3 30캡슐 30일분</t>
+          <t>콜라겐 60정 30일분</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1229,14 +1241,14 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000203&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000138&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>혈행</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1244,12 +1256,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>코엔자임 Q10 30캡슐 30일분</t>
+          <t>이지슬로 엑스트라버진 올리브오일＆레몬 4병</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>자연관</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1259,14 +1271,14 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000144&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=032627034&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1274,29 +1286,29 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>동국 맛있는 센시안 브이캔디 20정 20일분</t>
+          <t>[우형재 PICK] 익스트림 모노크레아틴 플러스 120 g 40일분</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>동국제약</t>
+          <t>익스트림</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3,000원</t>
+          <t>5,000원</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610910968&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=987253276&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>프로바이오틱스/유산균</t>
+          <t>비타민D</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1304,12 +1316,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>초코맛 생유산균 스틱 20포 20일분</t>
+          <t>비타민D＆아연 하루구미 30일분</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>유한양행</t>
+          <t>오브맘</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1319,14 +1331,14 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600651652&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=613602130&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>루테인/눈건강</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1334,7 +1346,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>녹차카테킨 30정 30일분</t>
+          <t>rTG 오메가3 30캡슐 30일분</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1349,14 +1361,14 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000136&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000145&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>비타민D</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1364,7 +1376,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>칼슘 마그네슘 비타민D 60정 30일분</t>
+          <t>쏘팔메토 옥타코사놀 30캡슐 30일분</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1379,7 +1391,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000148&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000139&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1406,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>[다영 PICK] 셀트리온 브로멜라인＆알파 CD 30정 15일분</t>
+          <t>동국 맛있는 센시안 브이캔디 20정 20일분</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1409,7 +1421,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=025575127&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610910968&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1436,32 +1448,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -1500,7 +1512,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1508,22 +1520,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>[7월 올영픽] 판도라 브이트리티 7/14포 (7/14일분)</t>
+          <t>프로뉴트리션 듀얼플랜 다이어트 유산균 14포</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>판도라</t>
+          <t>프로뉴트리션</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>24,500원</t>
+          <t>35,800원</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000227334&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=2</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000205496&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=2</t>
         </is>
       </c>
     </row>
@@ -1538,22 +1550,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>프로뉴트리션 듀얼플랜 다이어트 유산균 14포</t>
+          <t>[7월 올영픽/서현PICK] 콜레올로지 PRO 600mg*30(+10)/60정 단품</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>프로뉴트리션</t>
+          <t>푸드올로지</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>35,800원</t>
+          <t>14,900원</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000205496&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=3</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000175634&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=3</t>
         </is>
       </c>
     </row>
@@ -1568,29 +1580,29 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[골라담기] CJ웰케어 건강루틴 가격혁명 10종 택 1</t>
+          <t>[7월 올영픽] 식물성 멜라토닌 함유 멜라메이트 구미/로우슈가/버라이어티팩 구미 20/40/50구미</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>씨제이웰케어</t>
+          <t>멜라메이트</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>5,900원</t>
+          <t>13,000원</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000247861&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=4</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000223554&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=4</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>피부/미용</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1598,29 +1610,29 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>[7/2 단하루 1포 선착순 추가증정][7월 올영픽] 오니스트 트리플콜라겐 오렌지 14일 루틴</t>
+          <t>[NEW] 센트룸 이뮨부스트 데일리 프로텍션 C 14포 (14일분)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>오니스트</t>
+          <t>센트룸</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>28,900원</t>
+          <t>10,970원</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000188804&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=5</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000256462&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=5</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>피부/미용</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1628,29 +1640,29 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>[7월 올영픽] 에버콜라겐 스킨앤헤어 12포 기획 (+2포) (14일분)</t>
+          <t>[7월 올영픽] 콜레올로지 컷팅 젤리 레몬/키위/석류 10+2+2포 기획</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>에버콜라겐</t>
+          <t>푸드올로지</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>15,700원</t>
+          <t>18,100원</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000258818&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=6</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000183645&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=6</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>프로바이오틱스/유산균</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1658,22 +1670,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>[7월 올영픽/서현PICK] 콜레올로지 PRO 600mg*30(+10)/60정 단품</t>
+          <t>[덴프스] 덴마크 유산균이야기 우먼 2개월분(질유산균) + 철분 헤모케어 3포 증정</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>푸드올로지</t>
+          <t>덴프스</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>14,900원</t>
+          <t>37,050원</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000175634&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=7</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000202658&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=7</t>
         </is>
       </c>
     </row>
@@ -1718,29 +1730,29 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[7월 올영픽] 식물성 멜라토닌 함유 멜라메이트 구미/로우슈가/버라이어티팩 구미 20/40/50구미</t>
+          <t>코자아 식물성 멜라토닌 함유 젤리/드링크 (단품/기획)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>멜라메이트</t>
+          <t>코자아</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>13,000원</t>
+          <t>31,800원</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000223554&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=9</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000236755&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=9</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>프로바이오틱스/유산균</t>
+          <t>피부/미용</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1748,22 +1760,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>[포켓몬 에디션] 덴마크 유산균이야기 30캡슐 1+1 (+꼬부기 러기지택) (60일분)</t>
+          <t>[7/2 단하루 1포 선착순 추가증정][7월 올영픽] 오니스트 트리플콜라겐 오렌지 14일 루틴</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>덴프스</t>
+          <t>오니스트</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>30,400원</t>
+          <t>28,900원</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000206861&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=10</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000188804&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=10</t>
         </is>
       </c>
     </row>
@@ -1790,32 +1802,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>비율(%)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>카카오선물하기</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>다이소몰</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>올리브영</t>
         </is>
@@ -1894,16 +1906,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -1938,16 +1950,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -1960,16 +1972,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -1982,19 +1994,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C9" t="n">
-        <v>17.5</v>
+        <v>27.5</v>
       </c>
       <c r="D9" t="n">
         <v>5</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -2004,16 +2016,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
@@ -2035,10 +2047,10 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">

</xml_diff>